<commit_message>
Corregir columnas calculadas de la matriz de riesgos
Las celdas de formula se guardaban con un valor en cache vacio (<f>..</f><v/>)
y sin atributo de tipo. En las formulas que devuelven texto (columna L Nivel y
columna M Frecuencia) el tipo cacheado quedaba como numerico, por lo que varios
visores mostraban la celda en blanco aunque la formula estuviera presente.

Ahora cada celda de formula lleva su valor en cache con el tipo correcto
(t="str" para resultados de texto), en la matriz (K, L, M en las 118 filas) y en
el tablero (conteos, porcentajes y totales). Las formulas se conservan
intactas, asi que siguen recalculando al editar P e I.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DjaDU3QHWLpSnaydDxYzf7
</commit_message>
<xml_diff>
--- a/Checklist_Riesgos_Centro_Distribucion.xlsx
+++ b/Checklist_Riesgos_Centro_Distribucion.xlsx
@@ -3320,15 +3320,15 @@
       </c>
       <c r="K5" s="17">
         <f>IF(OR($I5="",$J5=""),"",$I5*$J5)</f>
-        <v/>
-      </c>
-      <c r="L5" s="17">
+        <v>10</v>
+      </c>
+      <c r="L5" s="17" t="str">
         <f>IF($K5="","",IF($K5&gt;=20,"Extremo",IF($K5&gt;=12,"Alto",IF($K5&gt;=6,"Medio",IF($K5&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M5" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M5" s="8" t="str">
         <f>IFERROR(VLOOKUP($L5,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
@@ -3399,15 +3399,15 @@
       </c>
       <c r="K6" s="17">
         <f>IF(OR($I6="",$J6=""),"",$I6*$J6)</f>
-        <v/>
-      </c>
-      <c r="L6" s="17">
+        <v>12</v>
+      </c>
+      <c r="L6" s="17" t="str">
         <f>IF($K6="","",IF($K6&gt;=20,"Extremo",IF($K6&gt;=12,"Alto",IF($K6&gt;=6,"Medio",IF($K6&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M6" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M6" s="8" t="str">
         <f>IFERROR(VLOOKUP($L6,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
@@ -3478,15 +3478,15 @@
       </c>
       <c r="K7" s="17">
         <f>IF(OR($I7="",$J7=""),"",$I7*$J7)</f>
-        <v/>
-      </c>
-      <c r="L7" s="17">
+        <v>12</v>
+      </c>
+      <c r="L7" s="17" t="str">
         <f>IF($K7="","",IF($K7&gt;=20,"Extremo",IF($K7&gt;=12,"Alto",IF($K7&gt;=6,"Medio",IF($K7&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M7" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M7" s="8" t="str">
         <f>IFERROR(VLOOKUP($L7,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
@@ -3557,15 +3557,15 @@
       </c>
       <c r="K8" s="17">
         <f>IF(OR($I8="",$J8=""),"",$I8*$J8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="17">
+        <v>15</v>
+      </c>
+      <c r="L8" s="17" t="str">
         <f>IF($K8="","",IF($K8&gt;=20,"Extremo",IF($K8&gt;=12,"Alto",IF($K8&gt;=6,"Medio",IF($K8&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M8" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M8" s="8" t="str">
         <f>IFERROR(VLOOKUP($L8,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
@@ -3636,15 +3636,15 @@
       </c>
       <c r="K9" s="17">
         <f>IF(OR($I9="",$J9=""),"",$I9*$J9)</f>
-        <v/>
-      </c>
-      <c r="L9" s="17">
+        <v>9</v>
+      </c>
+      <c r="L9" s="17" t="str">
         <f>IF($K9="","",IF($K9&gt;=20,"Extremo",IF($K9&gt;=12,"Alto",IF($K9&gt;=6,"Medio",IF($K9&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M9" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M9" s="8" t="str">
         <f>IFERROR(VLOOKUP($L9,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
@@ -3715,15 +3715,15 @@
       </c>
       <c r="K10" s="17">
         <f>IF(OR($I10="",$J10=""),"",$I10*$J10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="17">
+        <v>20</v>
+      </c>
+      <c r="L10" s="17" t="str">
         <f>IF($K10="","",IF($K10&gt;=20,"Extremo",IF($K10&gt;=12,"Alto",IF($K10&gt;=6,"Medio",IF($K10&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M10" s="8">
+        <v>Extremo</v>
+      </c>
+      <c r="M10" s="8" t="str">
         <f>IFERROR(VLOOKUP($L10,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Diaria o por turno (verificación operativa) + inspección formal semanal documentada</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
@@ -3794,15 +3794,15 @@
       </c>
       <c r="K11" s="17">
         <f>IF(OR($I11="",$J11=""),"",$I11*$J11)</f>
-        <v/>
-      </c>
-      <c r="L11" s="17">
+        <v>20</v>
+      </c>
+      <c r="L11" s="17" t="str">
         <f>IF($K11="","",IF($K11&gt;=20,"Extremo",IF($K11&gt;=12,"Alto",IF($K11&gt;=6,"Medio",IF($K11&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M11" s="8">
+        <v>Extremo</v>
+      </c>
+      <c r="M11" s="8" t="str">
         <f>IFERROR(VLOOKUP($L11,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Diaria o por turno (verificación operativa) + inspección formal semanal documentada</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
@@ -3873,15 +3873,15 @@
       </c>
       <c r="K12" s="17">
         <f>IF(OR($I12="",$J12=""),"",$I12*$J12)</f>
-        <v/>
-      </c>
-      <c r="L12" s="17">
+        <v>20</v>
+      </c>
+      <c r="L12" s="17" t="str">
         <f>IF($K12="","",IF($K12&gt;=20,"Extremo",IF($K12&gt;=12,"Alto",IF($K12&gt;=6,"Medio",IF($K12&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M12" s="8">
+        <v>Extremo</v>
+      </c>
+      <c r="M12" s="8" t="str">
         <f>IFERROR(VLOOKUP($L12,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Diaria o por turno (verificación operativa) + inspección formal semanal documentada</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
@@ -3952,15 +3952,15 @@
       </c>
       <c r="K13" s="17">
         <f>IF(OR($I13="",$J13=""),"",$I13*$J13)</f>
-        <v/>
-      </c>
-      <c r="L13" s="17">
+        <v>15</v>
+      </c>
+      <c r="L13" s="17" t="str">
         <f>IF($K13="","",IF($K13&gt;=20,"Extremo",IF($K13&gt;=12,"Alto",IF($K13&gt;=6,"Medio",IF($K13&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M13" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M13" s="8" t="str">
         <f>IFERROR(VLOOKUP($L13,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
@@ -4031,15 +4031,15 @@
       </c>
       <c r="K14" s="17">
         <f>IF(OR($I14="",$J14=""),"",$I14*$J14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="17">
+        <v>15</v>
+      </c>
+      <c r="L14" s="17" t="str">
         <f>IF($K14="","",IF($K14&gt;=20,"Extremo",IF($K14&gt;=12,"Alto",IF($K14&gt;=6,"Medio",IF($K14&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M14" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M14" s="8" t="str">
         <f>IFERROR(VLOOKUP($L14,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
@@ -4110,15 +4110,15 @@
       </c>
       <c r="K15" s="17">
         <f>IF(OR($I15="",$J15=""),"",$I15*$J15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="17">
+        <v>12</v>
+      </c>
+      <c r="L15" s="17" t="str">
         <f>IF($K15="","",IF($K15&gt;=20,"Extremo",IF($K15&gt;=12,"Alto",IF($K15&gt;=6,"Medio",IF($K15&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M15" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M15" s="8" t="str">
         <f>IFERROR(VLOOKUP($L15,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
@@ -4189,15 +4189,15 @@
       </c>
       <c r="K16" s="17">
         <f>IF(OR($I16="",$J16=""),"",$I16*$J16)</f>
-        <v/>
-      </c>
-      <c r="L16" s="17">
+        <v>15</v>
+      </c>
+      <c r="L16" s="17" t="str">
         <f>IF($K16="","",IF($K16&gt;=20,"Extremo",IF($K16&gt;=12,"Alto",IF($K16&gt;=6,"Medio",IF($K16&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M16" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M16" s="8" t="str">
         <f>IFERROR(VLOOKUP($L16,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
@@ -4268,15 +4268,15 @@
       </c>
       <c r="K17" s="17">
         <f>IF(OR($I17="",$J17=""),"",$I17*$J17)</f>
-        <v/>
-      </c>
-      <c r="L17" s="17">
+        <v>16</v>
+      </c>
+      <c r="L17" s="17" t="str">
         <f>IF($K17="","",IF($K17&gt;=20,"Extremo",IF($K17&gt;=12,"Alto",IF($K17&gt;=6,"Medio",IF($K17&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M17" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M17" s="8" t="str">
         <f>IFERROR(VLOOKUP($L17,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
@@ -4347,15 +4347,15 @@
       </c>
       <c r="K18" s="17">
         <f>IF(OR($I18="",$J18=""),"",$I18*$J18)</f>
-        <v/>
-      </c>
-      <c r="L18" s="17">
+        <v>15</v>
+      </c>
+      <c r="L18" s="17" t="str">
         <f>IF($K18="","",IF($K18&gt;=20,"Extremo",IF($K18&gt;=12,"Alto",IF($K18&gt;=6,"Medio",IF($K18&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M18" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M18" s="8" t="str">
         <f>IFERROR(VLOOKUP($L18,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
@@ -4426,15 +4426,15 @@
       </c>
       <c r="K19" s="17">
         <f>IF(OR($I19="",$J19=""),"",$I19*$J19)</f>
-        <v/>
-      </c>
-      <c r="L19" s="17">
+        <v>16</v>
+      </c>
+      <c r="L19" s="17" t="str">
         <f>IF($K19="","",IF($K19&gt;=20,"Extremo",IF($K19&gt;=12,"Alto",IF($K19&gt;=6,"Medio",IF($K19&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M19" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M19" s="8" t="str">
         <f>IFERROR(VLOOKUP($L19,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
@@ -4505,15 +4505,15 @@
       </c>
       <c r="K20" s="17">
         <f>IF(OR($I20="",$J20=""),"",$I20*$J20)</f>
-        <v/>
-      </c>
-      <c r="L20" s="17">
+        <v>16</v>
+      </c>
+      <c r="L20" s="17" t="str">
         <f>IF($K20="","",IF($K20&gt;=20,"Extremo",IF($K20&gt;=12,"Alto",IF($K20&gt;=6,"Medio",IF($K20&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M20" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M20" s="8" t="str">
         <f>IFERROR(VLOOKUP($L20,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
@@ -4584,15 +4584,15 @@
       </c>
       <c r="K21" s="17">
         <f>IF(OR($I21="",$J21=""),"",$I21*$J21)</f>
-        <v/>
-      </c>
-      <c r="L21" s="17">
+        <v>15</v>
+      </c>
+      <c r="L21" s="17" t="str">
         <f>IF($K21="","",IF($K21&gt;=20,"Extremo",IF($K21&gt;=12,"Alto",IF($K21&gt;=6,"Medio",IF($K21&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M21" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M21" s="8" t="str">
         <f>IFERROR(VLOOKUP($L21,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
@@ -4663,15 +4663,15 @@
       </c>
       <c r="K22" s="17">
         <f>IF(OR($I22="",$J22=""),"",$I22*$J22)</f>
-        <v/>
-      </c>
-      <c r="L22" s="17">
+        <v>10</v>
+      </c>
+      <c r="L22" s="17" t="str">
         <f>IF($K22="","",IF($K22&gt;=20,"Extremo",IF($K22&gt;=12,"Alto",IF($K22&gt;=6,"Medio",IF($K22&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M22" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M22" s="8" t="str">
         <f>IFERROR(VLOOKUP($L22,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
@@ -4742,15 +4742,15 @@
       </c>
       <c r="K23" s="17">
         <f>IF(OR($I23="",$J23=""),"",$I23*$J23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="17">
+        <v>16</v>
+      </c>
+      <c r="L23" s="17" t="str">
         <f>IF($K23="","",IF($K23&gt;=20,"Extremo",IF($K23&gt;=12,"Alto",IF($K23&gt;=6,"Medio",IF($K23&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M23" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M23" s="8" t="str">
         <f>IFERROR(VLOOKUP($L23,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
@@ -4821,15 +4821,15 @@
       </c>
       <c r="K24" s="17">
         <f>IF(OR($I24="",$J24=""),"",$I24*$J24)</f>
-        <v/>
-      </c>
-      <c r="L24" s="17">
+        <v>15</v>
+      </c>
+      <c r="L24" s="17" t="str">
         <f>IF($K24="","",IF($K24&gt;=20,"Extremo",IF($K24&gt;=12,"Alto",IF($K24&gt;=6,"Medio",IF($K24&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M24" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M24" s="8" t="str">
         <f>IFERROR(VLOOKUP($L24,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
@@ -4900,15 +4900,15 @@
       </c>
       <c r="K25" s="17">
         <f>IF(OR($I25="",$J25=""),"",$I25*$J25)</f>
-        <v/>
-      </c>
-      <c r="L25" s="17">
+        <v>20</v>
+      </c>
+      <c r="L25" s="17" t="str">
         <f>IF($K25="","",IF($K25&gt;=20,"Extremo",IF($K25&gt;=12,"Alto",IF($K25&gt;=6,"Medio",IF($K25&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M25" s="8">
+        <v>Extremo</v>
+      </c>
+      <c r="M25" s="8" t="str">
         <f>IFERROR(VLOOKUP($L25,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Diaria o por turno (verificación operativa) + inspección formal semanal documentada</v>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
@@ -4979,15 +4979,15 @@
       </c>
       <c r="K26" s="17">
         <f>IF(OR($I26="",$J26=""),"",$I26*$J26)</f>
-        <v/>
-      </c>
-      <c r="L26" s="17">
+        <v>10</v>
+      </c>
+      <c r="L26" s="17" t="str">
         <f>IF($K26="","",IF($K26&gt;=20,"Extremo",IF($K26&gt;=12,"Alto",IF($K26&gt;=6,"Medio",IF($K26&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M26" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M26" s="8" t="str">
         <f>IFERROR(VLOOKUP($L26,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
@@ -5058,15 +5058,15 @@
       </c>
       <c r="K27" s="17">
         <f>IF(OR($I27="",$J27=""),"",$I27*$J27)</f>
-        <v/>
-      </c>
-      <c r="L27" s="17">
+        <v>12</v>
+      </c>
+      <c r="L27" s="17" t="str">
         <f>IF($K27="","",IF($K27&gt;=20,"Extremo",IF($K27&gt;=12,"Alto",IF($K27&gt;=6,"Medio",IF($K27&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M27" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M27" s="8" t="str">
         <f>IFERROR(VLOOKUP($L27,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
@@ -5137,15 +5137,15 @@
       </c>
       <c r="K28" s="17">
         <f>IF(OR($I28="",$J28=""),"",$I28*$J28)</f>
-        <v/>
-      </c>
-      <c r="L28" s="17">
+        <v>12</v>
+      </c>
+      <c r="L28" s="17" t="str">
         <f>IF($K28="","",IF($K28&gt;=20,"Extremo",IF($K28&gt;=12,"Alto",IF($K28&gt;=6,"Medio",IF($K28&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M28" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M28" s="8" t="str">
         <f>IFERROR(VLOOKUP($L28,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
@@ -5216,15 +5216,15 @@
       </c>
       <c r="K29" s="17">
         <f>IF(OR($I29="",$J29=""),"",$I29*$J29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="17">
+        <v>15</v>
+      </c>
+      <c r="L29" s="17" t="str">
         <f>IF($K29="","",IF($K29&gt;=20,"Extremo",IF($K29&gt;=12,"Alto",IF($K29&gt;=6,"Medio",IF($K29&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M29" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M29" s="8" t="str">
         <f>IFERROR(VLOOKUP($L29,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
@@ -5295,15 +5295,15 @@
       </c>
       <c r="K30" s="17">
         <f>IF(OR($I30="",$J30=""),"",$I30*$J30)</f>
-        <v/>
-      </c>
-      <c r="L30" s="17">
+        <v>15</v>
+      </c>
+      <c r="L30" s="17" t="str">
         <f>IF($K30="","",IF($K30&gt;=20,"Extremo",IF($K30&gt;=12,"Alto",IF($K30&gt;=6,"Medio",IF($K30&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M30" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M30" s="8" t="str">
         <f>IFERROR(VLOOKUP($L30,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
@@ -5374,15 +5374,15 @@
       </c>
       <c r="K31" s="17">
         <f>IF(OR($I31="",$J31=""),"",$I31*$J31)</f>
-        <v/>
-      </c>
-      <c r="L31" s="17">
+        <v>12</v>
+      </c>
+      <c r="L31" s="17" t="str">
         <f>IF($K31="","",IF($K31&gt;=20,"Extremo",IF($K31&gt;=12,"Alto",IF($K31&gt;=6,"Medio",IF($K31&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M31" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M31" s="8" t="str">
         <f>IFERROR(VLOOKUP($L31,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
@@ -5453,15 +5453,15 @@
       </c>
       <c r="K32" s="17">
         <f>IF(OR($I32="",$J32=""),"",$I32*$J32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="17">
+        <v>9</v>
+      </c>
+      <c r="L32" s="17" t="str">
         <f>IF($K32="","",IF($K32&gt;=20,"Extremo",IF($K32&gt;=12,"Alto",IF($K32&gt;=6,"Medio",IF($K32&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M32" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M32" s="8" t="str">
         <f>IFERROR(VLOOKUP($L32,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
@@ -5532,15 +5532,15 @@
       </c>
       <c r="K33" s="17">
         <f>IF(OR($I33="",$J33=""),"",$I33*$J33)</f>
-        <v/>
-      </c>
-      <c r="L33" s="17">
+        <v>16</v>
+      </c>
+      <c r="L33" s="17" t="str">
         <f>IF($K33="","",IF($K33&gt;=20,"Extremo",IF($K33&gt;=12,"Alto",IF($K33&gt;=6,"Medio",IF($K33&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M33" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M33" s="8" t="str">
         <f>IFERROR(VLOOKUP($L33,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
@@ -5611,15 +5611,15 @@
       </c>
       <c r="K34" s="17">
         <f>IF(OR($I34="",$J34=""),"",$I34*$J34)</f>
-        <v/>
-      </c>
-      <c r="L34" s="17">
+        <v>12</v>
+      </c>
+      <c r="L34" s="17" t="str">
         <f>IF($K34="","",IF($K34&gt;=20,"Extremo",IF($K34&gt;=12,"Alto",IF($K34&gt;=6,"Medio",IF($K34&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M34" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M34" s="8" t="str">
         <f>IFERROR(VLOOKUP($L34,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
@@ -5690,15 +5690,15 @@
       </c>
       <c r="K35" s="17">
         <f>IF(OR($I35="",$J35=""),"",$I35*$J35)</f>
-        <v/>
-      </c>
-      <c r="L35" s="17">
+        <v>9</v>
+      </c>
+      <c r="L35" s="17" t="str">
         <f>IF($K35="","",IF($K35&gt;=20,"Extremo",IF($K35&gt;=12,"Alto",IF($K35&gt;=6,"Medio",IF($K35&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M35" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M35" s="8" t="str">
         <f>IFERROR(VLOOKUP($L35,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
@@ -5769,15 +5769,15 @@
       </c>
       <c r="K36" s="17">
         <f>IF(OR($I36="",$J36=""),"",$I36*$J36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="17">
+        <v>15</v>
+      </c>
+      <c r="L36" s="17" t="str">
         <f>IF($K36="","",IF($K36&gt;=20,"Extremo",IF($K36&gt;=12,"Alto",IF($K36&gt;=6,"Medio",IF($K36&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M36" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M36" s="8" t="str">
         <f>IFERROR(VLOOKUP($L36,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N36" s="8" t="inlineStr">
         <is>
@@ -5848,15 +5848,15 @@
       </c>
       <c r="K37" s="17">
         <f>IF(OR($I37="",$J37=""),"",$I37*$J37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="17">
+        <v>8</v>
+      </c>
+      <c r="L37" s="17" t="str">
         <f>IF($K37="","",IF($K37&gt;=20,"Extremo",IF($K37&gt;=12,"Alto",IF($K37&gt;=6,"Medio",IF($K37&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M37" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M37" s="8" t="str">
         <f>IFERROR(VLOOKUP($L37,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N37" s="8" t="inlineStr">
         <is>
@@ -5927,15 +5927,15 @@
       </c>
       <c r="K38" s="17">
         <f>IF(OR($I38="",$J38=""),"",$I38*$J38)</f>
-        <v/>
-      </c>
-      <c r="L38" s="17">
+        <v>9</v>
+      </c>
+      <c r="L38" s="17" t="str">
         <f>IF($K38="","",IF($K38&gt;=20,"Extremo",IF($K38&gt;=12,"Alto",IF($K38&gt;=6,"Medio",IF($K38&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M38" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M38" s="8" t="str">
         <f>IFERROR(VLOOKUP($L38,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N38" s="8" t="inlineStr">
         <is>
@@ -6006,15 +6006,15 @@
       </c>
       <c r="K39" s="17">
         <f>IF(OR($I39="",$J39=""),"",$I39*$J39)</f>
-        <v/>
-      </c>
-      <c r="L39" s="17">
+        <v>20</v>
+      </c>
+      <c r="L39" s="17" t="str">
         <f>IF($K39="","",IF($K39&gt;=20,"Extremo",IF($K39&gt;=12,"Alto",IF($K39&gt;=6,"Medio",IF($K39&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M39" s="8">
+        <v>Extremo</v>
+      </c>
+      <c r="M39" s="8" t="str">
         <f>IFERROR(VLOOKUP($L39,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Diaria o por turno (verificación operativa) + inspección formal semanal documentada</v>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
@@ -6085,15 +6085,15 @@
       </c>
       <c r="K40" s="17">
         <f>IF(OR($I40="",$J40=""),"",$I40*$J40)</f>
-        <v/>
-      </c>
-      <c r="L40" s="17">
+        <v>15</v>
+      </c>
+      <c r="L40" s="17" t="str">
         <f>IF($K40="","",IF($K40&gt;=20,"Extremo",IF($K40&gt;=12,"Alto",IF($K40&gt;=6,"Medio",IF($K40&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M40" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M40" s="8" t="str">
         <f>IFERROR(VLOOKUP($L40,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
@@ -6164,15 +6164,15 @@
       </c>
       <c r="K41" s="17">
         <f>IF(OR($I41="",$J41=""),"",$I41*$J41)</f>
-        <v/>
-      </c>
-      <c r="L41" s="17">
+        <v>15</v>
+      </c>
+      <c r="L41" s="17" t="str">
         <f>IF($K41="","",IF($K41&gt;=20,"Extremo",IF($K41&gt;=12,"Alto",IF($K41&gt;=6,"Medio",IF($K41&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M41" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M41" s="8" t="str">
         <f>IFERROR(VLOOKUP($L41,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N41" s="8" t="inlineStr">
         <is>
@@ -6243,15 +6243,15 @@
       </c>
       <c r="K42" s="17">
         <f>IF(OR($I42="",$J42=""),"",$I42*$J42)</f>
-        <v/>
-      </c>
-      <c r="L42" s="17">
+        <v>15</v>
+      </c>
+      <c r="L42" s="17" t="str">
         <f>IF($K42="","",IF($K42&gt;=20,"Extremo",IF($K42&gt;=12,"Alto",IF($K42&gt;=6,"Medio",IF($K42&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M42" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M42" s="8" t="str">
         <f>IFERROR(VLOOKUP($L42,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N42" s="8" t="inlineStr">
         <is>
@@ -6322,15 +6322,15 @@
       </c>
       <c r="K43" s="17">
         <f>IF(OR($I43="",$J43=""),"",$I43*$J43)</f>
-        <v/>
-      </c>
-      <c r="L43" s="17">
+        <v>15</v>
+      </c>
+      <c r="L43" s="17" t="str">
         <f>IF($K43="","",IF($K43&gt;=20,"Extremo",IF($K43&gt;=12,"Alto",IF($K43&gt;=6,"Medio",IF($K43&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M43" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M43" s="8" t="str">
         <f>IFERROR(VLOOKUP($L43,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N43" s="8" t="inlineStr">
         <is>
@@ -6401,15 +6401,15 @@
       </c>
       <c r="K44" s="17">
         <f>IF(OR($I44="",$J44=""),"",$I44*$J44)</f>
-        <v/>
-      </c>
-      <c r="L44" s="17">
+        <v>10</v>
+      </c>
+      <c r="L44" s="17" t="str">
         <f>IF($K44="","",IF($K44&gt;=20,"Extremo",IF($K44&gt;=12,"Alto",IF($K44&gt;=6,"Medio",IF($K44&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M44" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M44" s="8" t="str">
         <f>IFERROR(VLOOKUP($L44,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N44" s="8" t="inlineStr">
         <is>
@@ -6480,15 +6480,15 @@
       </c>
       <c r="K45" s="17">
         <f>IF(OR($I45="",$J45=""),"",$I45*$J45)</f>
-        <v/>
-      </c>
-      <c r="L45" s="17">
+        <v>15</v>
+      </c>
+      <c r="L45" s="17" t="str">
         <f>IF($K45="","",IF($K45&gt;=20,"Extremo",IF($K45&gt;=12,"Alto",IF($K45&gt;=6,"Medio",IF($K45&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M45" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M45" s="8" t="str">
         <f>IFERROR(VLOOKUP($L45,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N45" s="8" t="inlineStr">
         <is>
@@ -6559,15 +6559,15 @@
       </c>
       <c r="K46" s="17">
         <f>IF(OR($I46="",$J46=""),"",$I46*$J46)</f>
-        <v/>
-      </c>
-      <c r="L46" s="17">
+        <v>15</v>
+      </c>
+      <c r="L46" s="17" t="str">
         <f>IF($K46="","",IF($K46&gt;=20,"Extremo",IF($K46&gt;=12,"Alto",IF($K46&gt;=6,"Medio",IF($K46&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M46" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M46" s="8" t="str">
         <f>IFERROR(VLOOKUP($L46,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
@@ -6638,15 +6638,15 @@
       </c>
       <c r="K47" s="17">
         <f>IF(OR($I47="",$J47=""),"",$I47*$J47)</f>
-        <v/>
-      </c>
-      <c r="L47" s="17">
+        <v>15</v>
+      </c>
+      <c r="L47" s="17" t="str">
         <f>IF($K47="","",IF($K47&gt;=20,"Extremo",IF($K47&gt;=12,"Alto",IF($K47&gt;=6,"Medio",IF($K47&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M47" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M47" s="8" t="str">
         <f>IFERROR(VLOOKUP($L47,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N47" s="8" t="inlineStr">
         <is>
@@ -6717,15 +6717,15 @@
       </c>
       <c r="K48" s="17">
         <f>IF(OR($I48="",$J48=""),"",$I48*$J48)</f>
-        <v/>
-      </c>
-      <c r="L48" s="17">
+        <v>10</v>
+      </c>
+      <c r="L48" s="17" t="str">
         <f>IF($K48="","",IF($K48&gt;=20,"Extremo",IF($K48&gt;=12,"Alto",IF($K48&gt;=6,"Medio",IF($K48&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M48" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M48" s="8" t="str">
         <f>IFERROR(VLOOKUP($L48,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N48" s="8" t="inlineStr">
         <is>
@@ -6796,15 +6796,15 @@
       </c>
       <c r="K49" s="17">
         <f>IF(OR($I49="",$J49=""),"",$I49*$J49)</f>
-        <v/>
-      </c>
-      <c r="L49" s="17">
+        <v>10</v>
+      </c>
+      <c r="L49" s="17" t="str">
         <f>IF($K49="","",IF($K49&gt;=20,"Extremo",IF($K49&gt;=12,"Alto",IF($K49&gt;=6,"Medio",IF($K49&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M49" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M49" s="8" t="str">
         <f>IFERROR(VLOOKUP($L49,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
@@ -6875,15 +6875,15 @@
       </c>
       <c r="K50" s="17">
         <f>IF(OR($I50="",$J50=""),"",$I50*$J50)</f>
-        <v/>
-      </c>
-      <c r="L50" s="17">
+        <v>15</v>
+      </c>
+      <c r="L50" s="17" t="str">
         <f>IF($K50="","",IF($K50&gt;=20,"Extremo",IF($K50&gt;=12,"Alto",IF($K50&gt;=6,"Medio",IF($K50&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M50" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M50" s="8" t="str">
         <f>IFERROR(VLOOKUP($L50,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N50" s="8" t="inlineStr">
         <is>
@@ -6954,15 +6954,15 @@
       </c>
       <c r="K51" s="17">
         <f>IF(OR($I51="",$J51=""),"",$I51*$J51)</f>
-        <v/>
-      </c>
-      <c r="L51" s="17">
+        <v>15</v>
+      </c>
+      <c r="L51" s="17" t="str">
         <f>IF($K51="","",IF($K51&gt;=20,"Extremo",IF($K51&gt;=12,"Alto",IF($K51&gt;=6,"Medio",IF($K51&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M51" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M51" s="8" t="str">
         <f>IFERROR(VLOOKUP($L51,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
@@ -7033,15 +7033,15 @@
       </c>
       <c r="K52" s="17">
         <f>IF(OR($I52="",$J52=""),"",$I52*$J52)</f>
-        <v/>
-      </c>
-      <c r="L52" s="17">
+        <v>12</v>
+      </c>
+      <c r="L52" s="17" t="str">
         <f>IF($K52="","",IF($K52&gt;=20,"Extremo",IF($K52&gt;=12,"Alto",IF($K52&gt;=6,"Medio",IF($K52&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M52" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M52" s="8" t="str">
         <f>IFERROR(VLOOKUP($L52,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N52" s="8" t="inlineStr">
         <is>
@@ -7112,15 +7112,15 @@
       </c>
       <c r="K53" s="17">
         <f>IF(OR($I53="",$J53=""),"",$I53*$J53)</f>
-        <v/>
-      </c>
-      <c r="L53" s="17">
+        <v>15</v>
+      </c>
+      <c r="L53" s="17" t="str">
         <f>IF($K53="","",IF($K53&gt;=20,"Extremo",IF($K53&gt;=12,"Alto",IF($K53&gt;=6,"Medio",IF($K53&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M53" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M53" s="8" t="str">
         <f>IFERROR(VLOOKUP($L53,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
@@ -7191,15 +7191,15 @@
       </c>
       <c r="K54" s="17">
         <f>IF(OR($I54="",$J54=""),"",$I54*$J54)</f>
-        <v/>
-      </c>
-      <c r="L54" s="17">
+        <v>15</v>
+      </c>
+      <c r="L54" s="17" t="str">
         <f>IF($K54="","",IF($K54&gt;=20,"Extremo",IF($K54&gt;=12,"Alto",IF($K54&gt;=6,"Medio",IF($K54&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M54" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M54" s="8" t="str">
         <f>IFERROR(VLOOKUP($L54,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
@@ -7270,15 +7270,15 @@
       </c>
       <c r="K55" s="17">
         <f>IF(OR($I55="",$J55=""),"",$I55*$J55)</f>
-        <v/>
-      </c>
-      <c r="L55" s="17">
+        <v>15</v>
+      </c>
+      <c r="L55" s="17" t="str">
         <f>IF($K55="","",IF($K55&gt;=20,"Extremo",IF($K55&gt;=12,"Alto",IF($K55&gt;=6,"Medio",IF($K55&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M55" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M55" s="8" t="str">
         <f>IFERROR(VLOOKUP($L55,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N55" s="8" t="inlineStr">
         <is>
@@ -7349,15 +7349,15 @@
       </c>
       <c r="K56" s="17">
         <f>IF(OR($I56="",$J56=""),"",$I56*$J56)</f>
-        <v/>
-      </c>
-      <c r="L56" s="17">
+        <v>16</v>
+      </c>
+      <c r="L56" s="17" t="str">
         <f>IF($K56="","",IF($K56&gt;=20,"Extremo",IF($K56&gt;=12,"Alto",IF($K56&gt;=6,"Medio",IF($K56&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M56" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M56" s="8" t="str">
         <f>IFERROR(VLOOKUP($L56,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N56" s="8" t="inlineStr">
         <is>
@@ -7428,15 +7428,15 @@
       </c>
       <c r="K57" s="17">
         <f>IF(OR($I57="",$J57=""),"",$I57*$J57)</f>
-        <v/>
-      </c>
-      <c r="L57" s="17">
+        <v>16</v>
+      </c>
+      <c r="L57" s="17" t="str">
         <f>IF($K57="","",IF($K57&gt;=20,"Extremo",IF($K57&gt;=12,"Alto",IF($K57&gt;=6,"Medio",IF($K57&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M57" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M57" s="8" t="str">
         <f>IFERROR(VLOOKUP($L57,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N57" s="8" t="inlineStr">
         <is>
@@ -7507,15 +7507,15 @@
       </c>
       <c r="K58" s="17">
         <f>IF(OR($I58="",$J58=""),"",$I58*$J58)</f>
-        <v/>
-      </c>
-      <c r="L58" s="17">
+        <v>15</v>
+      </c>
+      <c r="L58" s="17" t="str">
         <f>IF($K58="","",IF($K58&gt;=20,"Extremo",IF($K58&gt;=12,"Alto",IF($K58&gt;=6,"Medio",IF($K58&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M58" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M58" s="8" t="str">
         <f>IFERROR(VLOOKUP($L58,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N58" s="8" t="inlineStr">
         <is>
@@ -7586,15 +7586,15 @@
       </c>
       <c r="K59" s="17">
         <f>IF(OR($I59="",$J59=""),"",$I59*$J59)</f>
-        <v/>
-      </c>
-      <c r="L59" s="17">
+        <v>15</v>
+      </c>
+      <c r="L59" s="17" t="str">
         <f>IF($K59="","",IF($K59&gt;=20,"Extremo",IF($K59&gt;=12,"Alto",IF($K59&gt;=6,"Medio",IF($K59&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M59" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M59" s="8" t="str">
         <f>IFERROR(VLOOKUP($L59,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N59" s="8" t="inlineStr">
         <is>
@@ -7665,15 +7665,15 @@
       </c>
       <c r="K60" s="17">
         <f>IF(OR($I60="",$J60=""),"",$I60*$J60)</f>
-        <v/>
-      </c>
-      <c r="L60" s="17">
+        <v>12</v>
+      </c>
+      <c r="L60" s="17" t="str">
         <f>IF($K60="","",IF($K60&gt;=20,"Extremo",IF($K60&gt;=12,"Alto",IF($K60&gt;=6,"Medio",IF($K60&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M60" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M60" s="8" t="str">
         <f>IFERROR(VLOOKUP($L60,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N60" s="8" t="inlineStr">
         <is>
@@ -7744,15 +7744,15 @@
       </c>
       <c r="K61" s="17">
         <f>IF(OR($I61="",$J61=""),"",$I61*$J61)</f>
-        <v/>
-      </c>
-      <c r="L61" s="17">
+        <v>15</v>
+      </c>
+      <c r="L61" s="17" t="str">
         <f>IF($K61="","",IF($K61&gt;=20,"Extremo",IF($K61&gt;=12,"Alto",IF($K61&gt;=6,"Medio",IF($K61&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M61" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M61" s="8" t="str">
         <f>IFERROR(VLOOKUP($L61,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N61" s="8" t="inlineStr">
         <is>
@@ -7823,15 +7823,15 @@
       </c>
       <c r="K62" s="17">
         <f>IF(OR($I62="",$J62=""),"",$I62*$J62)</f>
-        <v/>
-      </c>
-      <c r="L62" s="17">
+        <v>10</v>
+      </c>
+      <c r="L62" s="17" t="str">
         <f>IF($K62="","",IF($K62&gt;=20,"Extremo",IF($K62&gt;=12,"Alto",IF($K62&gt;=6,"Medio",IF($K62&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M62" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M62" s="8" t="str">
         <f>IFERROR(VLOOKUP($L62,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N62" s="8" t="inlineStr">
         <is>
@@ -7902,15 +7902,15 @@
       </c>
       <c r="K63" s="17">
         <f>IF(OR($I63="",$J63=""),"",$I63*$J63)</f>
-        <v/>
-      </c>
-      <c r="L63" s="17">
+        <v>15</v>
+      </c>
+      <c r="L63" s="17" t="str">
         <f>IF($K63="","",IF($K63&gt;=20,"Extremo",IF($K63&gt;=12,"Alto",IF($K63&gt;=6,"Medio",IF($K63&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M63" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M63" s="8" t="str">
         <f>IFERROR(VLOOKUP($L63,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N63" s="8" t="inlineStr">
         <is>
@@ -7981,15 +7981,15 @@
       </c>
       <c r="K64" s="17">
         <f>IF(OR($I64="",$J64=""),"",$I64*$J64)</f>
-        <v/>
-      </c>
-      <c r="L64" s="17">
+        <v>15</v>
+      </c>
+      <c r="L64" s="17" t="str">
         <f>IF($K64="","",IF($K64&gt;=20,"Extremo",IF($K64&gt;=12,"Alto",IF($K64&gt;=6,"Medio",IF($K64&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M64" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M64" s="8" t="str">
         <f>IFERROR(VLOOKUP($L64,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N64" s="8" t="inlineStr">
         <is>
@@ -8060,15 +8060,15 @@
       </c>
       <c r="K65" s="17">
         <f>IF(OR($I65="",$J65=""),"",$I65*$J65)</f>
-        <v/>
-      </c>
-      <c r="L65" s="17">
+        <v>15</v>
+      </c>
+      <c r="L65" s="17" t="str">
         <f>IF($K65="","",IF($K65&gt;=20,"Extremo",IF($K65&gt;=12,"Alto",IF($K65&gt;=6,"Medio",IF($K65&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M65" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M65" s="8" t="str">
         <f>IFERROR(VLOOKUP($L65,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N65" s="8" t="inlineStr">
         <is>
@@ -8139,15 +8139,15 @@
       </c>
       <c r="K66" s="17">
         <f>IF(OR($I66="",$J66=""),"",$I66*$J66)</f>
-        <v/>
-      </c>
-      <c r="L66" s="17">
+        <v>10</v>
+      </c>
+      <c r="L66" s="17" t="str">
         <f>IF($K66="","",IF($K66&gt;=20,"Extremo",IF($K66&gt;=12,"Alto",IF($K66&gt;=6,"Medio",IF($K66&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M66" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M66" s="8" t="str">
         <f>IFERROR(VLOOKUP($L66,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N66" s="8" t="inlineStr">
         <is>
@@ -8218,15 +8218,15 @@
       </c>
       <c r="K67" s="17">
         <f>IF(OR($I67="",$J67=""),"",$I67*$J67)</f>
-        <v/>
-      </c>
-      <c r="L67" s="17">
+        <v>8</v>
+      </c>
+      <c r="L67" s="17" t="str">
         <f>IF($K67="","",IF($K67&gt;=20,"Extremo",IF($K67&gt;=12,"Alto",IF($K67&gt;=6,"Medio",IF($K67&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M67" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M67" s="8" t="str">
         <f>IFERROR(VLOOKUP($L67,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N67" s="8" t="inlineStr">
         <is>
@@ -8297,15 +8297,15 @@
       </c>
       <c r="K68" s="17">
         <f>IF(OR($I68="",$J68=""),"",$I68*$J68)</f>
-        <v/>
-      </c>
-      <c r="L68" s="17">
+        <v>8</v>
+      </c>
+      <c r="L68" s="17" t="str">
         <f>IF($K68="","",IF($K68&gt;=20,"Extremo",IF($K68&gt;=12,"Alto",IF($K68&gt;=6,"Medio",IF($K68&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M68" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M68" s="8" t="str">
         <f>IFERROR(VLOOKUP($L68,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N68" s="8" t="inlineStr">
         <is>
@@ -8376,15 +8376,15 @@
       </c>
       <c r="K69" s="17">
         <f>IF(OR($I69="",$J69=""),"",$I69*$J69)</f>
-        <v/>
-      </c>
-      <c r="L69" s="17">
+        <v>8</v>
+      </c>
+      <c r="L69" s="17" t="str">
         <f>IF($K69="","",IF($K69&gt;=20,"Extremo",IF($K69&gt;=12,"Alto",IF($K69&gt;=6,"Medio",IF($K69&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M69" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M69" s="8" t="str">
         <f>IFERROR(VLOOKUP($L69,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N69" s="8" t="inlineStr">
         <is>
@@ -8455,15 +8455,15 @@
       </c>
       <c r="K70" s="17">
         <f>IF(OR($I70="",$J70=""),"",$I70*$J70)</f>
-        <v/>
-      </c>
-      <c r="L70" s="17">
+        <v>15</v>
+      </c>
+      <c r="L70" s="17" t="str">
         <f>IF($K70="","",IF($K70&gt;=20,"Extremo",IF($K70&gt;=12,"Alto",IF($K70&gt;=6,"Medio",IF($K70&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M70" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M70" s="8" t="str">
         <f>IFERROR(VLOOKUP($L70,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N70" s="8" t="inlineStr">
         <is>
@@ -8534,15 +8534,15 @@
       </c>
       <c r="K71" s="17">
         <f>IF(OR($I71="",$J71=""),"",$I71*$J71)</f>
-        <v/>
-      </c>
-      <c r="L71" s="17">
+        <v>15</v>
+      </c>
+      <c r="L71" s="17" t="str">
         <f>IF($K71="","",IF($K71&gt;=20,"Extremo",IF($K71&gt;=12,"Alto",IF($K71&gt;=6,"Medio",IF($K71&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M71" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M71" s="8" t="str">
         <f>IFERROR(VLOOKUP($L71,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N71" s="8" t="inlineStr">
         <is>
@@ -8613,15 +8613,15 @@
       </c>
       <c r="K72" s="17">
         <f>IF(OR($I72="",$J72=""),"",$I72*$J72)</f>
-        <v/>
-      </c>
-      <c r="L72" s="17">
+        <v>10</v>
+      </c>
+      <c r="L72" s="17" t="str">
         <f>IF($K72="","",IF($K72&gt;=20,"Extremo",IF($K72&gt;=12,"Alto",IF($K72&gt;=6,"Medio",IF($K72&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M72" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M72" s="8" t="str">
         <f>IFERROR(VLOOKUP($L72,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N72" s="8" t="inlineStr">
         <is>
@@ -8692,15 +8692,15 @@
       </c>
       <c r="K73" s="17">
         <f>IF(OR($I73="",$J73=""),"",$I73*$J73)</f>
-        <v/>
-      </c>
-      <c r="L73" s="17">
+        <v>12</v>
+      </c>
+      <c r="L73" s="17" t="str">
         <f>IF($K73="","",IF($K73&gt;=20,"Extremo",IF($K73&gt;=12,"Alto",IF($K73&gt;=6,"Medio",IF($K73&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M73" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M73" s="8" t="str">
         <f>IFERROR(VLOOKUP($L73,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N73" s="8" t="inlineStr">
         <is>
@@ -8771,15 +8771,15 @@
       </c>
       <c r="K74" s="17">
         <f>IF(OR($I74="",$J74=""),"",$I74*$J74)</f>
-        <v/>
-      </c>
-      <c r="L74" s="17">
+        <v>10</v>
+      </c>
+      <c r="L74" s="17" t="str">
         <f>IF($K74="","",IF($K74&gt;=20,"Extremo",IF($K74&gt;=12,"Alto",IF($K74&gt;=6,"Medio",IF($K74&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M74" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M74" s="8" t="str">
         <f>IFERROR(VLOOKUP($L74,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N74" s="8" t="inlineStr">
         <is>
@@ -8850,15 +8850,15 @@
       </c>
       <c r="K75" s="17">
         <f>IF(OR($I75="",$J75=""),"",$I75*$J75)</f>
-        <v/>
-      </c>
-      <c r="L75" s="17">
+        <v>6</v>
+      </c>
+      <c r="L75" s="17" t="str">
         <f>IF($K75="","",IF($K75&gt;=20,"Extremo",IF($K75&gt;=12,"Alto",IF($K75&gt;=6,"Medio",IF($K75&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M75" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M75" s="8" t="str">
         <f>IFERROR(VLOOKUP($L75,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N75" s="8" t="inlineStr">
         <is>
@@ -8929,15 +8929,15 @@
       </c>
       <c r="K76" s="17">
         <f>IF(OR($I76="",$J76=""),"",$I76*$J76)</f>
-        <v/>
-      </c>
-      <c r="L76" s="17">
+        <v>16</v>
+      </c>
+      <c r="L76" s="17" t="str">
         <f>IF($K76="","",IF($K76&gt;=20,"Extremo",IF($K76&gt;=12,"Alto",IF($K76&gt;=6,"Medio",IF($K76&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M76" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M76" s="8" t="str">
         <f>IFERROR(VLOOKUP($L76,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N76" s="8" t="inlineStr">
         <is>
@@ -9008,15 +9008,15 @@
       </c>
       <c r="K77" s="17">
         <f>IF(OR($I77="",$J77=""),"",$I77*$J77)</f>
-        <v/>
-      </c>
-      <c r="L77" s="17">
+        <v>10</v>
+      </c>
+      <c r="L77" s="17" t="str">
         <f>IF($K77="","",IF($K77&gt;=20,"Extremo",IF($K77&gt;=12,"Alto",IF($K77&gt;=6,"Medio",IF($K77&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M77" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M77" s="8" t="str">
         <f>IFERROR(VLOOKUP($L77,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N77" s="8" t="inlineStr">
         <is>
@@ -9087,15 +9087,15 @@
       </c>
       <c r="K78" s="17">
         <f>IF(OR($I78="",$J78=""),"",$I78*$J78)</f>
-        <v/>
-      </c>
-      <c r="L78" s="17">
+        <v>12</v>
+      </c>
+      <c r="L78" s="17" t="str">
         <f>IF($K78="","",IF($K78&gt;=20,"Extremo",IF($K78&gt;=12,"Alto",IF($K78&gt;=6,"Medio",IF($K78&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M78" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M78" s="8" t="str">
         <f>IFERROR(VLOOKUP($L78,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N78" s="8" t="inlineStr">
         <is>
@@ -9166,15 +9166,15 @@
       </c>
       <c r="K79" s="17">
         <f>IF(OR($I79="",$J79=""),"",$I79*$J79)</f>
-        <v/>
-      </c>
-      <c r="L79" s="17">
+        <v>12</v>
+      </c>
+      <c r="L79" s="17" t="str">
         <f>IF($K79="","",IF($K79&gt;=20,"Extremo",IF($K79&gt;=12,"Alto",IF($K79&gt;=6,"Medio",IF($K79&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M79" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M79" s="8" t="str">
         <f>IFERROR(VLOOKUP($L79,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N79" s="8" t="inlineStr">
         <is>
@@ -9245,15 +9245,15 @@
       </c>
       <c r="K80" s="17">
         <f>IF(OR($I80="",$J80=""),"",$I80*$J80)</f>
-        <v/>
-      </c>
-      <c r="L80" s="17">
+        <v>10</v>
+      </c>
+      <c r="L80" s="17" t="str">
         <f>IF($K80="","",IF($K80&gt;=20,"Extremo",IF($K80&gt;=12,"Alto",IF($K80&gt;=6,"Medio",IF($K80&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M80" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M80" s="8" t="str">
         <f>IFERROR(VLOOKUP($L80,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N80" s="8" t="inlineStr">
         <is>
@@ -9324,15 +9324,15 @@
       </c>
       <c r="K81" s="17">
         <f>IF(OR($I81="",$J81=""),"",$I81*$J81)</f>
-        <v/>
-      </c>
-      <c r="L81" s="17">
+        <v>12</v>
+      </c>
+      <c r="L81" s="17" t="str">
         <f>IF($K81="","",IF($K81&gt;=20,"Extremo",IF($K81&gt;=12,"Alto",IF($K81&gt;=6,"Medio",IF($K81&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M81" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M81" s="8" t="str">
         <f>IFERROR(VLOOKUP($L81,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N81" s="8" t="inlineStr">
         <is>
@@ -9403,15 +9403,15 @@
       </c>
       <c r="K82" s="17">
         <f>IF(OR($I82="",$J82=""),"",$I82*$J82)</f>
-        <v/>
-      </c>
-      <c r="L82" s="17">
+        <v>12</v>
+      </c>
+      <c r="L82" s="17" t="str">
         <f>IF($K82="","",IF($K82&gt;=20,"Extremo",IF($K82&gt;=12,"Alto",IF($K82&gt;=6,"Medio",IF($K82&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M82" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M82" s="8" t="str">
         <f>IFERROR(VLOOKUP($L82,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N82" s="8" t="inlineStr">
         <is>
@@ -9482,15 +9482,15 @@
       </c>
       <c r="K83" s="17">
         <f>IF(OR($I83="",$J83=""),"",$I83*$J83)</f>
-        <v/>
-      </c>
-      <c r="L83" s="17">
+        <v>10</v>
+      </c>
+      <c r="L83" s="17" t="str">
         <f>IF($K83="","",IF($K83&gt;=20,"Extremo",IF($K83&gt;=12,"Alto",IF($K83&gt;=6,"Medio",IF($K83&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M83" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M83" s="8" t="str">
         <f>IFERROR(VLOOKUP($L83,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N83" s="8" t="inlineStr">
         <is>
@@ -9561,15 +9561,15 @@
       </c>
       <c r="K84" s="17">
         <f>IF(OR($I84="",$J84=""),"",$I84*$J84)</f>
-        <v/>
-      </c>
-      <c r="L84" s="17">
+        <v>15</v>
+      </c>
+      <c r="L84" s="17" t="str">
         <f>IF($K84="","",IF($K84&gt;=20,"Extremo",IF($K84&gt;=12,"Alto",IF($K84&gt;=6,"Medio",IF($K84&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M84" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M84" s="8" t="str">
         <f>IFERROR(VLOOKUP($L84,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N84" s="8" t="inlineStr">
         <is>
@@ -9640,15 +9640,15 @@
       </c>
       <c r="K85" s="17">
         <f>IF(OR($I85="",$J85=""),"",$I85*$J85)</f>
-        <v/>
-      </c>
-      <c r="L85" s="17">
+        <v>15</v>
+      </c>
+      <c r="L85" s="17" t="str">
         <f>IF($K85="","",IF($K85&gt;=20,"Extremo",IF($K85&gt;=12,"Alto",IF($K85&gt;=6,"Medio",IF($K85&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M85" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M85" s="8" t="str">
         <f>IFERROR(VLOOKUP($L85,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N85" s="8" t="inlineStr">
         <is>
@@ -9719,15 +9719,15 @@
       </c>
       <c r="K86" s="17">
         <f>IF(OR($I86="",$J86=""),"",$I86*$J86)</f>
-        <v/>
-      </c>
-      <c r="L86" s="17">
+        <v>9</v>
+      </c>
+      <c r="L86" s="17" t="str">
         <f>IF($K86="","",IF($K86&gt;=20,"Extremo",IF($K86&gt;=12,"Alto",IF($K86&gt;=6,"Medio",IF($K86&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M86" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M86" s="8" t="str">
         <f>IFERROR(VLOOKUP($L86,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N86" s="8" t="inlineStr">
         <is>
@@ -9798,15 +9798,15 @@
       </c>
       <c r="K87" s="17">
         <f>IF(OR($I87="",$J87=""),"",$I87*$J87)</f>
-        <v/>
-      </c>
-      <c r="L87" s="17">
+        <v>12</v>
+      </c>
+      <c r="L87" s="17" t="str">
         <f>IF($K87="","",IF($K87&gt;=20,"Extremo",IF($K87&gt;=12,"Alto",IF($K87&gt;=6,"Medio",IF($K87&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M87" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M87" s="8" t="str">
         <f>IFERROR(VLOOKUP($L87,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N87" s="8" t="inlineStr">
         <is>
@@ -9877,15 +9877,15 @@
       </c>
       <c r="K88" s="17">
         <f>IF(OR($I88="",$J88=""),"",$I88*$J88)</f>
-        <v/>
-      </c>
-      <c r="L88" s="17">
+        <v>12</v>
+      </c>
+      <c r="L88" s="17" t="str">
         <f>IF($K88="","",IF($K88&gt;=20,"Extremo",IF($K88&gt;=12,"Alto",IF($K88&gt;=6,"Medio",IF($K88&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M88" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M88" s="8" t="str">
         <f>IFERROR(VLOOKUP($L88,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N88" s="8" t="inlineStr">
         <is>
@@ -9956,15 +9956,15 @@
       </c>
       <c r="K89" s="17">
         <f>IF(OR($I89="",$J89=""),"",$I89*$J89)</f>
-        <v/>
-      </c>
-      <c r="L89" s="17">
+        <v>12</v>
+      </c>
+      <c r="L89" s="17" t="str">
         <f>IF($K89="","",IF($K89&gt;=20,"Extremo",IF($K89&gt;=12,"Alto",IF($K89&gt;=6,"Medio",IF($K89&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M89" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M89" s="8" t="str">
         <f>IFERROR(VLOOKUP($L89,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N89" s="8" t="inlineStr">
         <is>
@@ -10035,15 +10035,15 @@
       </c>
       <c r="K90" s="17">
         <f>IF(OR($I90="",$J90=""),"",$I90*$J90)</f>
-        <v/>
-      </c>
-      <c r="L90" s="17">
+        <v>15</v>
+      </c>
+      <c r="L90" s="17" t="str">
         <f>IF($K90="","",IF($K90&gt;=20,"Extremo",IF($K90&gt;=12,"Alto",IF($K90&gt;=6,"Medio",IF($K90&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M90" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M90" s="8" t="str">
         <f>IFERROR(VLOOKUP($L90,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N90" s="8" t="inlineStr">
         <is>
@@ -10114,15 +10114,15 @@
       </c>
       <c r="K91" s="17">
         <f>IF(OR($I91="",$J91=""),"",$I91*$J91)</f>
-        <v/>
-      </c>
-      <c r="L91" s="17">
+        <v>9</v>
+      </c>
+      <c r="L91" s="17" t="str">
         <f>IF($K91="","",IF($K91&gt;=20,"Extremo",IF($K91&gt;=12,"Alto",IF($K91&gt;=6,"Medio",IF($K91&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M91" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M91" s="8" t="str">
         <f>IFERROR(VLOOKUP($L91,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N91" s="8" t="inlineStr">
         <is>
@@ -10193,15 +10193,15 @@
       </c>
       <c r="K92" s="17">
         <f>IF(OR($I92="",$J92=""),"",$I92*$J92)</f>
-        <v/>
-      </c>
-      <c r="L92" s="17">
+        <v>9</v>
+      </c>
+      <c r="L92" s="17" t="str">
         <f>IF($K92="","",IF($K92&gt;=20,"Extremo",IF($K92&gt;=12,"Alto",IF($K92&gt;=6,"Medio",IF($K92&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M92" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M92" s="8" t="str">
         <f>IFERROR(VLOOKUP($L92,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N92" s="8" t="inlineStr">
         <is>
@@ -10272,15 +10272,15 @@
       </c>
       <c r="K93" s="17">
         <f>IF(OR($I93="",$J93=""),"",$I93*$J93)</f>
-        <v/>
-      </c>
-      <c r="L93" s="17">
+        <v>16</v>
+      </c>
+      <c r="L93" s="17" t="str">
         <f>IF($K93="","",IF($K93&gt;=20,"Extremo",IF($K93&gt;=12,"Alto",IF($K93&gt;=6,"Medio",IF($K93&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M93" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M93" s="8" t="str">
         <f>IFERROR(VLOOKUP($L93,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N93" s="8" t="inlineStr">
         <is>
@@ -10351,15 +10351,15 @@
       </c>
       <c r="K94" s="17">
         <f>IF(OR($I94="",$J94=""),"",$I94*$J94)</f>
-        <v/>
-      </c>
-      <c r="L94" s="17">
+        <v>9</v>
+      </c>
+      <c r="L94" s="17" t="str">
         <f>IF($K94="","",IF($K94&gt;=20,"Extremo",IF($K94&gt;=12,"Alto",IF($K94&gt;=6,"Medio",IF($K94&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M94" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M94" s="8" t="str">
         <f>IFERROR(VLOOKUP($L94,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N94" s="8" t="inlineStr">
         <is>
@@ -10430,15 +10430,15 @@
       </c>
       <c r="K95" s="17">
         <f>IF(OR($I95="",$J95=""),"",$I95*$J95)</f>
-        <v/>
-      </c>
-      <c r="L95" s="17">
+        <v>10</v>
+      </c>
+      <c r="L95" s="17" t="str">
         <f>IF($K95="","",IF($K95&gt;=20,"Extremo",IF($K95&gt;=12,"Alto",IF($K95&gt;=6,"Medio",IF($K95&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M95" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M95" s="8" t="str">
         <f>IFERROR(VLOOKUP($L95,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N95" s="8" t="inlineStr">
         <is>
@@ -10509,15 +10509,15 @@
       </c>
       <c r="K96" s="17">
         <f>IF(OR($I96="",$J96=""),"",$I96*$J96)</f>
-        <v/>
-      </c>
-      <c r="L96" s="17">
+        <v>12</v>
+      </c>
+      <c r="L96" s="17" t="str">
         <f>IF($K96="","",IF($K96&gt;=20,"Extremo",IF($K96&gt;=12,"Alto",IF($K96&gt;=6,"Medio",IF($K96&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M96" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M96" s="8" t="str">
         <f>IFERROR(VLOOKUP($L96,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N96" s="8" t="inlineStr">
         <is>
@@ -10588,15 +10588,15 @@
       </c>
       <c r="K97" s="17">
         <f>IF(OR($I97="",$J97=""),"",$I97*$J97)</f>
-        <v/>
-      </c>
-      <c r="L97" s="17">
+        <v>15</v>
+      </c>
+      <c r="L97" s="17" t="str">
         <f>IF($K97="","",IF($K97&gt;=20,"Extremo",IF($K97&gt;=12,"Alto",IF($K97&gt;=6,"Medio",IF($K97&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M97" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M97" s="8" t="str">
         <f>IFERROR(VLOOKUP($L97,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N97" s="8" t="inlineStr">
         <is>
@@ -10667,15 +10667,15 @@
       </c>
       <c r="K98" s="17">
         <f>IF(OR($I98="",$J98=""),"",$I98*$J98)</f>
-        <v/>
-      </c>
-      <c r="L98" s="17">
+        <v>12</v>
+      </c>
+      <c r="L98" s="17" t="str">
         <f>IF($K98="","",IF($K98&gt;=20,"Extremo",IF($K98&gt;=12,"Alto",IF($K98&gt;=6,"Medio",IF($K98&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M98" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M98" s="8" t="str">
         <f>IFERROR(VLOOKUP($L98,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N98" s="8" t="inlineStr">
         <is>
@@ -10746,15 +10746,15 @@
       </c>
       <c r="K99" s="17">
         <f>IF(OR($I99="",$J99=""),"",$I99*$J99)</f>
-        <v/>
-      </c>
-      <c r="L99" s="17">
+        <v>15</v>
+      </c>
+      <c r="L99" s="17" t="str">
         <f>IF($K99="","",IF($K99&gt;=20,"Extremo",IF($K99&gt;=12,"Alto",IF($K99&gt;=6,"Medio",IF($K99&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M99" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M99" s="8" t="str">
         <f>IFERROR(VLOOKUP($L99,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N99" s="8" t="inlineStr">
         <is>
@@ -10825,15 +10825,15 @@
       </c>
       <c r="K100" s="17">
         <f>IF(OR($I100="",$J100=""),"",$I100*$J100)</f>
-        <v/>
-      </c>
-      <c r="L100" s="17">
+        <v>12</v>
+      </c>
+      <c r="L100" s="17" t="str">
         <f>IF($K100="","",IF($K100&gt;=20,"Extremo",IF($K100&gt;=12,"Alto",IF($K100&gt;=6,"Medio",IF($K100&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M100" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M100" s="8" t="str">
         <f>IFERROR(VLOOKUP($L100,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N100" s="8" t="inlineStr">
         <is>
@@ -10904,15 +10904,15 @@
       </c>
       <c r="K101" s="17">
         <f>IF(OR($I101="",$J101=""),"",$I101*$J101)</f>
-        <v/>
-      </c>
-      <c r="L101" s="17">
+        <v>15</v>
+      </c>
+      <c r="L101" s="17" t="str">
         <f>IF($K101="","",IF($K101&gt;=20,"Extremo",IF($K101&gt;=12,"Alto",IF($K101&gt;=6,"Medio",IF($K101&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M101" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M101" s="8" t="str">
         <f>IFERROR(VLOOKUP($L101,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N101" s="8" t="inlineStr">
         <is>
@@ -10983,15 +10983,15 @@
       </c>
       <c r="K102" s="17">
         <f>IF(OR($I102="",$J102=""),"",$I102*$J102)</f>
-        <v/>
-      </c>
-      <c r="L102" s="17">
+        <v>9</v>
+      </c>
+      <c r="L102" s="17" t="str">
         <f>IF($K102="","",IF($K102&gt;=20,"Extremo",IF($K102&gt;=12,"Alto",IF($K102&gt;=6,"Medio",IF($K102&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M102" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M102" s="8" t="str">
         <f>IFERROR(VLOOKUP($L102,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N102" s="8" t="inlineStr">
         <is>
@@ -11062,15 +11062,15 @@
       </c>
       <c r="K103" s="17">
         <f>IF(OR($I103="",$J103=""),"",$I103*$J103)</f>
-        <v/>
-      </c>
-      <c r="L103" s="17">
+        <v>12</v>
+      </c>
+      <c r="L103" s="17" t="str">
         <f>IF($K103="","",IF($K103&gt;=20,"Extremo",IF($K103&gt;=12,"Alto",IF($K103&gt;=6,"Medio",IF($K103&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M103" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M103" s="8" t="str">
         <f>IFERROR(VLOOKUP($L103,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N103" s="8" t="inlineStr">
         <is>
@@ -11141,15 +11141,15 @@
       </c>
       <c r="K104" s="17">
         <f>IF(OR($I104="",$J104=""),"",$I104*$J104)</f>
-        <v/>
-      </c>
-      <c r="L104" s="17">
+        <v>12</v>
+      </c>
+      <c r="L104" s="17" t="str">
         <f>IF($K104="","",IF($K104&gt;=20,"Extremo",IF($K104&gt;=12,"Alto",IF($K104&gt;=6,"Medio",IF($K104&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M104" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M104" s="8" t="str">
         <f>IFERROR(VLOOKUP($L104,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N104" s="8" t="inlineStr">
         <is>
@@ -11220,15 +11220,15 @@
       </c>
       <c r="K105" s="17">
         <f>IF(OR($I105="",$J105=""),"",$I105*$J105)</f>
-        <v/>
-      </c>
-      <c r="L105" s="17">
+        <v>9</v>
+      </c>
+      <c r="L105" s="17" t="str">
         <f>IF($K105="","",IF($K105&gt;=20,"Extremo",IF($K105&gt;=12,"Alto",IF($K105&gt;=6,"Medio",IF($K105&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M105" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M105" s="8" t="str">
         <f>IFERROR(VLOOKUP($L105,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N105" s="8" t="inlineStr">
         <is>
@@ -11299,15 +11299,15 @@
       </c>
       <c r="K106" s="17">
         <f>IF(OR($I106="",$J106=""),"",$I106*$J106)</f>
-        <v/>
-      </c>
-      <c r="L106" s="17">
+        <v>10</v>
+      </c>
+      <c r="L106" s="17" t="str">
         <f>IF($K106="","",IF($K106&gt;=20,"Extremo",IF($K106&gt;=12,"Alto",IF($K106&gt;=6,"Medio",IF($K106&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M106" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M106" s="8" t="str">
         <f>IFERROR(VLOOKUP($L106,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N106" s="8" t="inlineStr">
         <is>
@@ -11378,15 +11378,15 @@
       </c>
       <c r="K107" s="17">
         <f>IF(OR($I107="",$J107=""),"",$I107*$J107)</f>
-        <v/>
-      </c>
-      <c r="L107" s="17">
+        <v>12</v>
+      </c>
+      <c r="L107" s="17" t="str">
         <f>IF($K107="","",IF($K107&gt;=20,"Extremo",IF($K107&gt;=12,"Alto",IF($K107&gt;=6,"Medio",IF($K107&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M107" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M107" s="8" t="str">
         <f>IFERROR(VLOOKUP($L107,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N107" s="8" t="inlineStr">
         <is>
@@ -11457,15 +11457,15 @@
       </c>
       <c r="K108" s="17">
         <f>IF(OR($I108="",$J108=""),"",$I108*$J108)</f>
-        <v/>
-      </c>
-      <c r="L108" s="17">
+        <v>9</v>
+      </c>
+      <c r="L108" s="17" t="str">
         <f>IF($K108="","",IF($K108&gt;=20,"Extremo",IF($K108&gt;=12,"Alto",IF($K108&gt;=6,"Medio",IF($K108&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M108" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M108" s="8" t="str">
         <f>IFERROR(VLOOKUP($L108,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N108" s="8" t="inlineStr">
         <is>
@@ -11536,15 +11536,15 @@
       </c>
       <c r="K109" s="17">
         <f>IF(OR($I109="",$J109=""),"",$I109*$J109)</f>
-        <v/>
-      </c>
-      <c r="L109" s="17">
+        <v>9</v>
+      </c>
+      <c r="L109" s="17" t="str">
         <f>IF($K109="","",IF($K109&gt;=20,"Extremo",IF($K109&gt;=12,"Alto",IF($K109&gt;=6,"Medio",IF($K109&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M109" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M109" s="8" t="str">
         <f>IFERROR(VLOOKUP($L109,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N109" s="8" t="inlineStr">
         <is>
@@ -11615,15 +11615,15 @@
       </c>
       <c r="K110" s="17">
         <f>IF(OR($I110="",$J110=""),"",$I110*$J110)</f>
-        <v/>
-      </c>
-      <c r="L110" s="17">
+        <v>9</v>
+      </c>
+      <c r="L110" s="17" t="str">
         <f>IF($K110="","",IF($K110&gt;=20,"Extremo",IF($K110&gt;=12,"Alto",IF($K110&gt;=6,"Medio",IF($K110&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M110" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M110" s="8" t="str">
         <f>IFERROR(VLOOKUP($L110,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N110" s="8" t="inlineStr">
         <is>
@@ -11694,15 +11694,15 @@
       </c>
       <c r="K111" s="17">
         <f>IF(OR($I111="",$J111=""),"",$I111*$J111)</f>
-        <v/>
-      </c>
-      <c r="L111" s="17">
+        <v>9</v>
+      </c>
+      <c r="L111" s="17" t="str">
         <f>IF($K111="","",IF($K111&gt;=20,"Extremo",IF($K111&gt;=12,"Alto",IF($K111&gt;=6,"Medio",IF($K111&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M111" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M111" s="8" t="str">
         <f>IFERROR(VLOOKUP($L111,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N111" s="8" t="inlineStr">
         <is>
@@ -11773,15 +11773,15 @@
       </c>
       <c r="K112" s="17">
         <f>IF(OR($I112="",$J112=""),"",$I112*$J112)</f>
-        <v/>
-      </c>
-      <c r="L112" s="17">
+        <v>15</v>
+      </c>
+      <c r="L112" s="17" t="str">
         <f>IF($K112="","",IF($K112&gt;=20,"Extremo",IF($K112&gt;=12,"Alto",IF($K112&gt;=6,"Medio",IF($K112&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M112" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M112" s="8" t="str">
         <f>IFERROR(VLOOKUP($L112,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N112" s="8" t="inlineStr">
         <is>
@@ -11852,15 +11852,15 @@
       </c>
       <c r="K113" s="17">
         <f>IF(OR($I113="",$J113=""),"",$I113*$J113)</f>
-        <v/>
-      </c>
-      <c r="L113" s="17">
+        <v>10</v>
+      </c>
+      <c r="L113" s="17" t="str">
         <f>IF($K113="","",IF($K113&gt;=20,"Extremo",IF($K113&gt;=12,"Alto",IF($K113&gt;=6,"Medio",IF($K113&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M113" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M113" s="8" t="str">
         <f>IFERROR(VLOOKUP($L113,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N113" s="8" t="inlineStr">
         <is>
@@ -11931,15 +11931,15 @@
       </c>
       <c r="K114" s="17">
         <f>IF(OR($I114="",$J114=""),"",$I114*$J114)</f>
-        <v/>
-      </c>
-      <c r="L114" s="17">
+        <v>12</v>
+      </c>
+      <c r="L114" s="17" t="str">
         <f>IF($K114="","",IF($K114&gt;=20,"Extremo",IF($K114&gt;=12,"Alto",IF($K114&gt;=6,"Medio",IF($K114&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M114" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M114" s="8" t="str">
         <f>IFERROR(VLOOKUP($L114,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N114" s="8" t="inlineStr">
         <is>
@@ -12010,15 +12010,15 @@
       </c>
       <c r="K115" s="17">
         <f>IF(OR($I115="",$J115=""),"",$I115*$J115)</f>
-        <v/>
-      </c>
-      <c r="L115" s="17">
+        <v>12</v>
+      </c>
+      <c r="L115" s="17" t="str">
         <f>IF($K115="","",IF($K115&gt;=20,"Extremo",IF($K115&gt;=12,"Alto",IF($K115&gt;=6,"Medio",IF($K115&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M115" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M115" s="8" t="str">
         <f>IFERROR(VLOOKUP($L115,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N115" s="8" t="inlineStr">
         <is>
@@ -12089,15 +12089,15 @@
       </c>
       <c r="K116" s="17">
         <f>IF(OR($I116="",$J116=""),"",$I116*$J116)</f>
-        <v/>
-      </c>
-      <c r="L116" s="17">
+        <v>10</v>
+      </c>
+      <c r="L116" s="17" t="str">
         <f>IF($K116="","",IF($K116&gt;=20,"Extremo",IF($K116&gt;=12,"Alto",IF($K116&gt;=6,"Medio",IF($K116&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M116" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M116" s="8" t="str">
         <f>IFERROR(VLOOKUP($L116,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N116" s="8" t="inlineStr">
         <is>
@@ -12168,15 +12168,15 @@
       </c>
       <c r="K117" s="17">
         <f>IF(OR($I117="",$J117=""),"",$I117*$J117)</f>
-        <v/>
-      </c>
-      <c r="L117" s="17">
+        <v>10</v>
+      </c>
+      <c r="L117" s="17" t="str">
         <f>IF($K117="","",IF($K117&gt;=20,"Extremo",IF($K117&gt;=12,"Alto",IF($K117&gt;=6,"Medio",IF($K117&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M117" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M117" s="8" t="str">
         <f>IFERROR(VLOOKUP($L117,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N117" s="8" t="inlineStr">
         <is>
@@ -12247,15 +12247,15 @@
       </c>
       <c r="K118" s="17">
         <f>IF(OR($I118="",$J118=""),"",$I118*$J118)</f>
-        <v/>
-      </c>
-      <c r="L118" s="17">
+        <v>12</v>
+      </c>
+      <c r="L118" s="17" t="str">
         <f>IF($K118="","",IF($K118&gt;=20,"Extremo",IF($K118&gt;=12,"Alto",IF($K118&gt;=6,"Medio",IF($K118&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M118" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M118" s="8" t="str">
         <f>IFERROR(VLOOKUP($L118,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N118" s="8" t="inlineStr">
         <is>
@@ -12326,15 +12326,15 @@
       </c>
       <c r="K119" s="17">
         <f>IF(OR($I119="",$J119=""),"",$I119*$J119)</f>
-        <v/>
-      </c>
-      <c r="L119" s="17">
+        <v>15</v>
+      </c>
+      <c r="L119" s="17" t="str">
         <f>IF($K119="","",IF($K119&gt;=20,"Extremo",IF($K119&gt;=12,"Alto",IF($K119&gt;=6,"Medio",IF($K119&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M119" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M119" s="8" t="str">
         <f>IFERROR(VLOOKUP($L119,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N119" s="8" t="inlineStr">
         <is>
@@ -12405,15 +12405,15 @@
       </c>
       <c r="K120" s="17">
         <f>IF(OR($I120="",$J120=""),"",$I120*$J120)</f>
-        <v/>
-      </c>
-      <c r="L120" s="17">
+        <v>10</v>
+      </c>
+      <c r="L120" s="17" t="str">
         <f>IF($K120="","",IF($K120&gt;=20,"Extremo",IF($K120&gt;=12,"Alto",IF($K120&gt;=6,"Medio",IF($K120&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M120" s="8">
+        <v>Medio</v>
+      </c>
+      <c r="M120" s="8" t="str">
         <f>IFERROR(VLOOKUP($L120,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Mensual para elementos operativos; trimestral para elementos estructurales o de instalación</v>
       </c>
       <c r="N120" s="8" t="inlineStr">
         <is>
@@ -12484,15 +12484,15 @@
       </c>
       <c r="K121" s="17">
         <f>IF(OR($I121="",$J121=""),"",$I121*$J121)</f>
-        <v/>
-      </c>
-      <c r="L121" s="17">
+        <v>12</v>
+      </c>
+      <c r="L121" s="17" t="str">
         <f>IF($K121="","",IF($K121&gt;=20,"Extremo",IF($K121&gt;=12,"Alto",IF($K121&gt;=6,"Medio",IF($K121&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M121" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M121" s="8" t="str">
         <f>IFERROR(VLOOKUP($L121,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N121" s="8" t="inlineStr">
         <is>
@@ -12563,15 +12563,15 @@
       </c>
       <c r="K122" s="17">
         <f>IF(OR($I122="",$J122=""),"",$I122*$J122)</f>
-        <v/>
-      </c>
-      <c r="L122" s="17">
+        <v>12</v>
+      </c>
+      <c r="L122" s="17" t="str">
         <f>IF($K122="","",IF($K122&gt;=20,"Extremo",IF($K122&gt;=12,"Alto",IF($K122&gt;=6,"Medio",IF($K122&gt;=3,"Bajo","Muy bajo")))))</f>
-        <v/>
-      </c>
-      <c r="M122" s="8">
+        <v>Alto</v>
+      </c>
+      <c r="M122" s="8" t="str">
         <f>IFERROR(VLOOKUP($L122,'3. Escalas y Criterios'!$A$30:$C$34,3,FALSE),"")</f>
-        <v/>
+        <v>Semanal (verificación) + inspección formal mensual documentada</v>
       </c>
       <c r="N122" s="8" t="inlineStr">
         <is>
@@ -18607,11 +18607,11 @@
       </c>
       <c r="C6" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="D6" s="47">
         <f>IFERROR(C6/$C$11,0)</f>
-        <v/>
+        <v>0.0423728813559322</v>
       </c>
       <c r="E6" s="48" t="inlineStr">
         <is>
@@ -18631,11 +18631,11 @@
       </c>
       <c r="C7" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="D7" s="47">
         <f>IFERROR(C7/$C$11,0)</f>
-        <v/>
+        <v>0.635593220338983</v>
       </c>
       <c r="E7" s="48" t="inlineStr">
         <is>
@@ -18655,11 +18655,11 @@
       </c>
       <c r="C8" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D8" s="47">
         <f>IFERROR(C8/$C$11,0)</f>
-        <v/>
+        <v>0.3220338983050847</v>
       </c>
       <c r="E8" s="48" t="inlineStr">
         <is>
@@ -18679,11 +18679,11 @@
       </c>
       <c r="C9" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D9" s="47">
         <f>IFERROR(C9/$C$11,0)</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E9" s="48" t="inlineStr">
         <is>
@@ -18703,11 +18703,11 @@
       </c>
       <c r="C10" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D10" s="47">
         <f>IFERROR(C10/$C$11,0)</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E10" s="48" t="inlineStr">
         <is>
@@ -18727,7 +18727,7 @@
       </c>
       <c r="C11" s="50">
         <f>SUM(C6:C10)</f>
-        <v/>
+        <v>118</v>
       </c>
       <c r="D11" s="51" t="n"/>
     </row>
@@ -18769,11 +18769,11 @@
       </c>
       <c r="C15" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$Q$5:$Q$122,"Sí")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D15" s="47">
         <f>IFERROR(C15/COUNTA('2. Matriz de Riesgos'!$Q$5:$Q$122),0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -18784,11 +18784,11 @@
       </c>
       <c r="C16" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$Q$5:$Q$122,"Parcial")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D16" s="47">
         <f>IFERROR(C16/COUNTA('2. Matriz de Riesgos'!$Q$5:$Q$122),0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -18799,11 +18799,11 @@
       </c>
       <c r="C17" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$Q$5:$Q$122,"No")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D17" s="47">
         <f>IFERROR(C17/COUNTA('2. Matriz de Riesgos'!$Q$5:$Q$122),0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -18814,11 +18814,11 @@
       </c>
       <c r="C18" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$Q$5:$Q$122,"N.A.")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D18" s="47">
         <f>IFERROR(C18/COUNTA('2. Matriz de Riesgos'!$Q$5:$Q$122),0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -18829,11 +18829,11 @@
       </c>
       <c r="C19" s="46">
         <f>COUNTIF('2. Matriz de Riesgos'!$Q$5:$Q$122,"Sin evaluar")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D19" s="47">
         <f>IFERROR(C19/COUNTA('2. Matriz de Riesgos'!$Q$5:$Q$122),0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -18844,7 +18844,7 @@
       </c>
       <c r="C20" s="52">
         <f>IFERROR(C15/(C15+C16+C17),0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D20" s="51" t="n"/>
     </row>
@@ -18906,31 +18906,31 @@
       </c>
       <c r="C24" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B24,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="D24" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B24,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="E24" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B24,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F24" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B24,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G24" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B24,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H24" s="17">
         <f>SUM(C24:G24)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="I24" s="46">
         <f>C24+D24</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
@@ -18941,31 +18941,31 @@
       </c>
       <c r="C25" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B25,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D25" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B25,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E25" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B25,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F25" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B25,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G25" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B25,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H25" s="17">
         <f>SUM(C25:G25)</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="I25" s="46">
         <f>C25+D25</f>
-        <v/>
+        <v>11</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -18976,31 +18976,31 @@
       </c>
       <c r="C26" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B26,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="D26" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B26,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="E26" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B26,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F26" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B26,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G26" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B26,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H26" s="17">
         <f>SUM(C26:G26)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="I26" s="46">
         <f>C26+D26</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -19011,31 +19011,31 @@
       </c>
       <c r="C27" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B27,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D27" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B27,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="E27" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B27,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F27" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B27,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G27" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B27,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H27" s="17">
         <f>SUM(C27:G27)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="I27" s="46">
         <f>C27+D27</f>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -19046,31 +19046,31 @@
       </c>
       <c r="C28" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B28,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="D28" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B28,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="E28" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B28,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F28" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B28,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G28" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B28,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H28" s="17">
         <f>SUM(C28:G28)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="I28" s="46">
         <f>C28+D28</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
@@ -19081,31 +19081,31 @@
       </c>
       <c r="C29" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B29,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D29" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B29,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="E29" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B29,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F29" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B29,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G29" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B29,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H29" s="17">
         <f>SUM(C29:G29)</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="I29" s="46">
         <f>C29+D29</f>
-        <v/>
+        <v>12</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -19116,31 +19116,31 @@
       </c>
       <c r="C30" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B30,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D30" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B30,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="E30" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B30,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="F30" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B30,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G30" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B30,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H30" s="17">
         <f>SUM(C30:G30)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="I30" s="46">
         <f>C30+D30</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -19151,31 +19151,31 @@
       </c>
       <c r="C31" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B31,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D31" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B31,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E31" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B31,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F31" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B31,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G31" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B31,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H31" s="17">
         <f>SUM(C31:G31)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I31" s="46">
         <f>C31+D31</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
@@ -19186,31 +19186,31 @@
       </c>
       <c r="C32" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B32,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D32" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B32,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="E32" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B32,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F32" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B32,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G32" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B32,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H32" s="17">
         <f>SUM(C32:G32)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="I32" s="46">
         <f>C32+D32</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -19221,31 +19221,31 @@
       </c>
       <c r="C33" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B33,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D33" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B33,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="E33" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B33,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F33" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B33,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G33" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B33,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H33" s="17">
         <f>SUM(C33:G33)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I33" s="46">
         <f>C33+D33</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
@@ -19256,31 +19256,31 @@
       </c>
       <c r="C34" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B34,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D34" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B34,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="E34" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B34,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F34" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B34,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G34" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B34,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H34" s="17">
         <f>SUM(C34:G34)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="I34" s="46">
         <f>C34+D34</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -19291,31 +19291,31 @@
       </c>
       <c r="C35" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B35,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D35" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B35,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="E35" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B35,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F35" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B35,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G35" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B35,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H35" s="17">
         <f>SUM(C35:G35)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="I35" s="46">
         <f>C35+D35</f>
-        <v/>
+        <v>7</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -19326,31 +19326,31 @@
       </c>
       <c r="C36" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B36,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D36" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B36,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="E36" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B36,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F36" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B36,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G36" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B36,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H36" s="17">
         <f>SUM(C36:G36)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I36" s="46">
         <f>C36+D36</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
@@ -19361,31 +19361,31 @@
       </c>
       <c r="C37" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B37,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D37" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B37,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="E37" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B37,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F37" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B37,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G37" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B37,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H37" s="17">
         <f>SUM(C37:G37)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I37" s="46">
         <f>C37+D37</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -19396,31 +19396,31 @@
       </c>
       <c r="C38" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B38,'2. Matriz de Riesgos'!$L$5:$L$122,"Extremo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D38" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B38,'2. Matriz de Riesgos'!$L$5:$L$122,"Alto")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="E38" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B38,'2. Matriz de Riesgos'!$L$5:$L$122,"Medio")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F38" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B38,'2. Matriz de Riesgos'!$L$5:$L$122,"Bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G38" s="46">
         <f>COUNTIFS('2. Matriz de Riesgos'!$B$5:$B$122,$B38,'2. Matriz de Riesgos'!$L$5:$L$122,"Muy bajo")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H38" s="17">
         <f>SUM(C38:G38)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="I38" s="46">
         <f>C38+D38</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Corregir formato condicional que ocultaba el texto de la columna Nivel
En un formato diferencial (dxf) Excel pinta el fondo de la celda con bgColor,
no con fgColor. Las reglas se escribieron con fgColor, de modo que el relleno
nunca se aplicaba pero el color de letra si: los niveles Extremo, Alto y Bajo
quedaban en letra blanca sobre fondo blanco y la celda parecia vacia, mientras
Medio y Muy bajo (letra negra) si se veian. El mismo defecto afectaba a la
columna Cumple y a los estados del plan de accion.

Ahora todas las reglas usan bgColor con tinte claro y letra oscura, legible
incluso si un visor ignora el relleno. Ninguna regla usa letra blanca.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DjaDU3QHWLpSnaydDxYzf7
</commit_message>
<xml_diff>
--- a/Checklist_Riesgos_Centro_Distribucion.xlsx
+++ b/Checklist_Riesgos_Centro_Distribucion.xlsx
@@ -450,104 +450,98 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C00000"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FF974706"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00ED7D31"/>
+        <patternFill>
+          <bgColor rgb="FFFCD5B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00000000"/>
+        <color rgb="FF9C6500"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC000"/>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="0070AD47"/>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="00000000"/>
+        <color rgb="FF3F3F3F"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00BFBFBF"/>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F4B7B7"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F8CBAD"/>
+        <patternFill>
+          <bgColor rgb="FFFCD5B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFE699"/>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC000"/>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
+        <color rgb="FF1F3864"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F4B7B7"/>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -18506,12 +18500,15 @@
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Cerrada"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Abierta"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="9">
+      <formula>"En ejecución"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H44">
-    <cfRule type="expression" priority="4" dxfId="5">
+    <cfRule type="expression" priority="5" dxfId="0">
       <formula>AND($H5&lt;&gt;"",$I5="",$H5&lt;TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19824,12 +19821,12 @@
     <mergeCell ref="C49:D49"/>
   </mergeCells>
   <conditionalFormatting sqref="C24:C38">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="10">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24:D38">
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>